<commit_message>
Mark leetcode 2824 done
</commit_message>
<xml_diff>
--- a/7.Patterns Practice.xlsx
+++ b/7.Patterns Practice.xlsx
@@ -1,26 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29127"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\samyak\learning\java\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC1036FE-FDA3-4B97-90B1-21948588E779}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Two Pointers" sheetId="1" r:id="rId1"/>
+    <sheet r:id="rId1" sheetId="1" name="Two Pointers"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="60">
   <si>
     <t>No.</t>
   </si>
@@ -207,7 +201,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
+  <numFmts count="0"/>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -220,14 +215,14 @@
       <sz val="13"/>
       <color rgb="FF000000"/>
       <name val="Comic Sans MS"/>
-      <family val="4"/>
+      <family val="2"/>
     </font>
     <font>
       <u/>
       <sz val="13"/>
       <color rgb="FF000000"/>
       <name val="Comic Sans MS"/>
-      <family val="4"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="5">
@@ -239,17 +234,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFBBC04"/>
+        <fgColor rgb="FFfbbc04"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF00FF00"/>
+        <fgColor rgb="FF00ff00"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFFF"/>
+        <fgColor rgb="FFffffff"/>
       </patternFill>
     </fill>
   </fills>
@@ -263,16 +258,16 @@
     </border>
     <border>
       <left style="medium">
-        <color rgb="FFCCCCCC"/>
+        <color rgb="FFcccccc"/>
       </left>
       <right style="medium">
-        <color rgb="FFCCCCCC"/>
+        <color rgb="FFcccccc"/>
       </right>
       <top style="medium">
-        <color rgb="FFCCCCCC"/>
+        <color rgb="FFcccccc"/>
       </top>
       <bottom style="medium">
-        <color rgb="FFCCCCCC"/>
+        <color rgb="FFcccccc"/>
       </bottom>
       <diagonal/>
     </border>
@@ -281,58 +276,55 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="14">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle xfId="0" builtinId="0" name="Normal"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    <ext uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14ac:slicerStyles xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -343,10 +335,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
+        <a:sysClr lastClr="000000" val="windowText"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
+        <a:sysClr lastClr="FFFFFF" val="window"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="44546A"/>
@@ -384,71 +376,71 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
+        <a:font typeface="맑은 고딕" script="Hang"/>
+        <a:font typeface="宋体" script="Hans"/>
+        <a:font typeface="新細明體" script="Hant"/>
+        <a:font typeface="Times New Roman" script="Arab"/>
+        <a:font typeface="Times New Roman" script="Hebr"/>
+        <a:font typeface="Tahoma" script="Thai"/>
+        <a:font typeface="Nyala" script="Ethi"/>
+        <a:font typeface="Vrinda" script="Beng"/>
+        <a:font typeface="Shruti" script="Gujr"/>
+        <a:font typeface="MoolBoran" script="Khmr"/>
+        <a:font typeface="Tunga" script="Knda"/>
+        <a:font typeface="Raavi" script="Guru"/>
+        <a:font typeface="Euphemia" script="Cans"/>
+        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
+        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
+        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
+        <a:font typeface="MV Boli" script="Thaa"/>
+        <a:font typeface="Mangal" script="Deva"/>
+        <a:font typeface="Gautami" script="Telu"/>
+        <a:font typeface="Latha" script="Taml"/>
+        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
+        <a:font typeface="Kalinga" script="Orya"/>
+        <a:font typeface="Kartika" script="Mlym"/>
+        <a:font typeface="DokChampa" script="Laoo"/>
+        <a:font typeface="Iskoola Pota" script="Sinh"/>
+        <a:font typeface="Mongolian Baiti" script="Mong"/>
+        <a:font typeface="Times New Roman" script="Viet"/>
+        <a:font typeface="Microsoft Uighur" script="Uigh"/>
+        <a:font typeface="Sylfaen" script="Geor"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
+        <a:font typeface="맑은 고딕" script="Hang"/>
+        <a:font typeface="宋体" script="Hans"/>
+        <a:font typeface="新細明體" script="Hant"/>
+        <a:font typeface="Arial" script="Arab"/>
+        <a:font typeface="Arial" script="Hebr"/>
+        <a:font typeface="Tahoma" script="Thai"/>
+        <a:font typeface="Nyala" script="Ethi"/>
+        <a:font typeface="Vrinda" script="Beng"/>
+        <a:font typeface="Shruti" script="Gujr"/>
+        <a:font typeface="DaunPenh" script="Khmr"/>
+        <a:font typeface="Tunga" script="Knda"/>
+        <a:font typeface="Raavi" script="Guru"/>
+        <a:font typeface="Euphemia" script="Cans"/>
+        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
+        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
+        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
+        <a:font typeface="MV Boli" script="Thaa"/>
+        <a:font typeface="Mangal" script="Deva"/>
+        <a:font typeface="Gautami" script="Telu"/>
+        <a:font typeface="Latha" script="Taml"/>
+        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
+        <a:font typeface="Kalinga" script="Orya"/>
+        <a:font typeface="Kartika" script="Mlym"/>
+        <a:font typeface="DokChampa" script="Laoo"/>
+        <a:font typeface="Iskoola Pota" script="Sinh"/>
+        <a:font typeface="Mongolian Baiti" script="Mong"/>
+        <a:font typeface="Arial" script="Viet"/>
+        <a:font typeface="Microsoft Uighur" script="Uigh"/>
+        <a:font typeface="Sylfaen" script="Geor"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -476,7 +468,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
+          <a:lin scaled="1" ang="16200000"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
@@ -499,11 +491,11 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
+          <a:lin scaled="1" ang="16200000"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cmpd="sng" cap="flat" w="9525">
           <a:solidFill>
             <a:schemeClr val="phClr">
               <a:shade val="9500"/>
@@ -512,13 +504,13 @@
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cmpd="sng" cap="flat" w="25400">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cmpd="sng" cap="flat" w="38100">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -528,7 +520,7 @@
       <a:effectStyleLst>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
               <a:srgbClr val="000000">
                 <a:alpha val="38000"/>
               </a:srgbClr>
@@ -537,7 +529,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -546,7 +538,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -554,10 +546,10 @@
           </a:effectLst>
           <a:scene3d>
             <a:camera prst="orthographicFront">
-              <a:rot lat="0" lon="0" rev="0"/>
+              <a:rot rev="0" lon="0" lat="0"/>
             </a:camera>
-            <a:lightRig rig="threePt" dir="t">
-              <a:rot lat="0" lon="0" rev="1200000"/>
+            <a:lightRig dir="t" rig="threePt">
+              <a:rot rev="1200000" lon="0" lat="0"/>
             </a:lightRig>
           </a:scene3d>
           <a:sp3d>
@@ -622,505 +614,509 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:G24"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="5.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="68.21875" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.88671875" style="2" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="121.77734375" style="2" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="7" style="2" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" style="12" width="5.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="13" width="16.14785714285714" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="13" width="68.29071428571429" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="13" width="9.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="13" width="121.7192857142857" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="13" width="7.005" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="12" width="9.719285714285713" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="19.8" x14ac:dyDescent="0.45">
-      <c r="A1" s="9" t="s">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="21.75">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="10" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="10" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="10" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="9" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="19.8" x14ac:dyDescent="0.45">
-      <c r="A2" s="11">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="21.75">
+      <c r="A2" s="3">
         <v>1</v>
       </c>
-      <c r="B2" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C2" s="3" t="s">
+      <c r="B2" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="F2" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="G2" s="11">
+      <c r="G2" s="3">
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="19.8" x14ac:dyDescent="0.45">
-      <c r="A3" s="11">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="21.75">
+      <c r="A3" s="3">
         <v>2</v>
       </c>
-      <c r="B3" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C3" s="3" t="s">
+      <c r="B3" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="E3" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="F3" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="G3" s="11">
+      <c r="G3" s="3">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="19.8" x14ac:dyDescent="0.45">
-      <c r="A4" s="11">
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="21.75">
+      <c r="A4" s="3">
         <v>3</v>
       </c>
-      <c r="B4" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C4" s="3" t="s">
+      <c r="B4" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="E4" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="F4" s="3"/>
-      <c r="G4" s="11"/>
-    </row>
-    <row r="5" spans="1:7" ht="19.8" x14ac:dyDescent="0.45">
-      <c r="A5" s="11">
+      <c r="F4" s="4"/>
+      <c r="G4" s="3"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="21.75">
+      <c r="A5" s="3">
         <v>4</v>
       </c>
-      <c r="B5" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C5" s="3" t="s">
+      <c r="B5" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="E5" s="6" t="s">
+      <c r="E5" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="F5" s="3"/>
-      <c r="G5" s="11"/>
-    </row>
-    <row r="6" spans="1:7" ht="19.8" x14ac:dyDescent="0.45">
-      <c r="A6" s="11">
+      <c r="F5" s="4"/>
+      <c r="G5" s="3"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="21.75">
+      <c r="A6" s="3">
         <v>5</v>
       </c>
-      <c r="B6" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C6" s="3" t="s">
+      <c r="B6" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C6" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="E6" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="F6" s="3"/>
-      <c r="G6" s="11"/>
-    </row>
-    <row r="7" spans="1:7" ht="19.8" x14ac:dyDescent="0.45">
-      <c r="A7" s="11">
+      <c r="F6" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G6" s="3"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="21.75">
+      <c r="A7" s="3">
         <v>6</v>
       </c>
-      <c r="B7" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C7" s="3" t="s">
+      <c r="B7" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C7" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="D7" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="E7" s="6" t="s">
+      <c r="E7" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="F7" s="3"/>
-      <c r="G7" s="11"/>
-    </row>
-    <row r="8" spans="1:7" ht="19.8" x14ac:dyDescent="0.45">
-      <c r="A8" s="12">
-        <v>7</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="C8" s="4" t="s">
+      <c r="F7" s="4"/>
+      <c r="G7" s="3"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="21.75">
+      <c r="A8" s="6">
+        <v>7</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C8" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="D8" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="E8" s="7" t="s">
+      <c r="E8" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="F8" s="4"/>
-      <c r="G8" s="12"/>
-    </row>
-    <row r="9" spans="1:7" ht="19.8" x14ac:dyDescent="0.45">
-      <c r="A9" s="12">
+      <c r="F8" s="7"/>
+      <c r="G8" s="6"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="21.75">
+      <c r="A9" s="6">
         <v>8</v>
       </c>
-      <c r="B9" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="C9" s="4" t="s">
+      <c r="B9" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C9" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="D9" s="4" t="s">
+      <c r="D9" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="E9" s="7" t="s">
+      <c r="E9" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="F9" s="4"/>
-      <c r="G9" s="12"/>
-    </row>
-    <row r="10" spans="1:7" ht="19.8" x14ac:dyDescent="0.45">
-      <c r="A10" s="12">
+      <c r="F9" s="7"/>
+      <c r="G9" s="6"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="21.75">
+      <c r="A10" s="6">
         <v>9</v>
       </c>
-      <c r="B10" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="C10" s="4" t="s">
+      <c r="B10" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C10" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="D10" s="4" t="s">
+      <c r="D10" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="E10" s="7" t="s">
+      <c r="E10" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="F10" s="4"/>
-      <c r="G10" s="12"/>
-    </row>
-    <row r="11" spans="1:7" ht="19.8" x14ac:dyDescent="0.45">
-      <c r="A11" s="12">
+      <c r="F10" s="7"/>
+      <c r="G10" s="6"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="21.75">
+      <c r="A11" s="6">
         <v>10</v>
       </c>
-      <c r="B11" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="C11" s="4" t="s">
+      <c r="B11" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C11" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="D11" s="4" t="s">
+      <c r="D11" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="E11" s="7" t="s">
+      <c r="E11" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="F11" s="4"/>
-      <c r="G11" s="12"/>
-    </row>
-    <row r="12" spans="1:7" ht="19.8" x14ac:dyDescent="0.45">
-      <c r="A12" s="11">
+      <c r="F11" s="7"/>
+      <c r="G11" s="6"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="21.75">
+      <c r="A12" s="3">
         <v>11</v>
       </c>
-      <c r="B12" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C12" s="3" t="s">
+      <c r="B12" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C12" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="D12" s="3" t="s">
+      <c r="D12" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="E12" s="6" t="s">
+      <c r="E12" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="F12" s="3" t="s">
+      <c r="F12" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="G12" s="11">
+      <c r="G12" s="3">
         <v>2</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="19.8" x14ac:dyDescent="0.45">
-      <c r="A13" s="11">
+    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="17.25">
+      <c r="A13" s="3">
         <v>12</v>
       </c>
-      <c r="B13" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C13" s="3" t="s">
+      <c r="B13" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C13" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="D13" s="3" t="s">
+      <c r="D13" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="E13" s="6" t="s">
+      <c r="E13" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="F13" s="3"/>
-      <c r="G13" s="11"/>
-    </row>
-    <row r="14" spans="1:7" ht="19.8" x14ac:dyDescent="0.45">
-      <c r="A14" s="13">
+      <c r="F13" s="4"/>
+      <c r="G13" s="3"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="17.25">
+      <c r="A14" s="9">
         <v>13</v>
       </c>
-      <c r="B14" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="C14" s="5" t="s">
+      <c r="B14" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C14" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="D14" s="5" t="s">
+      <c r="D14" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="E14" s="8" t="s">
+      <c r="E14" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="F14" s="5"/>
-      <c r="G14" s="13"/>
-    </row>
-    <row r="15" spans="1:7" ht="19.8" x14ac:dyDescent="0.45">
-      <c r="A15" s="11">
+      <c r="F14" s="10"/>
+      <c r="G14" s="9"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="17.25">
+      <c r="A15" s="3">
         <v>14</v>
       </c>
-      <c r="B15" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C15" s="3" t="s">
+      <c r="B15" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C15" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="D15" s="3" t="s">
+      <c r="D15" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="E15" s="6" t="s">
+      <c r="E15" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="F15" s="3"/>
-      <c r="G15" s="11"/>
-    </row>
-    <row r="16" spans="1:7" ht="19.8" x14ac:dyDescent="0.45">
-      <c r="A16" s="13">
+      <c r="F15" s="4"/>
+      <c r="G15" s="3"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="17.25">
+      <c r="A16" s="9">
         <v>15</v>
       </c>
-      <c r="B16" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="C16" s="5" t="s">
+      <c r="B16" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C16" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="D16" s="5" t="s">
+      <c r="D16" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="E16" s="8" t="s">
+      <c r="E16" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="F16" s="5"/>
-      <c r="G16" s="13"/>
-    </row>
-    <row r="17" spans="1:7" ht="19.8" x14ac:dyDescent="0.45">
-      <c r="A17" s="11">
+      <c r="F16" s="10"/>
+      <c r="G16" s="9"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="17.25">
+      <c r="A17" s="3">
         <v>16</v>
       </c>
-      <c r="B17" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C17" s="3" t="s">
+      <c r="B17" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C17" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="D17" s="3" t="s">
+      <c r="D17" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="E17" s="6" t="s">
+      <c r="E17" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="F17" s="3"/>
-      <c r="G17" s="11"/>
-    </row>
-    <row r="18" spans="1:7" ht="19.8" x14ac:dyDescent="0.45">
-      <c r="A18" s="11">
+      <c r="F17" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G17" s="3"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="17.25">
+      <c r="A18" s="3">
         <v>17</v>
       </c>
-      <c r="B18" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C18" s="3" t="s">
+      <c r="B18" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C18" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="D18" s="3" t="s">
+      <c r="D18" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="E18" s="6" t="s">
+      <c r="E18" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="F18" s="3" t="s">
+      <c r="F18" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="G18" s="11">
+      <c r="G18" s="3">
         <v>2</v>
       </c>
     </row>
-    <row r="19" spans="1:7" ht="19.8" x14ac:dyDescent="0.45">
-      <c r="A19" s="11">
+    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="17.25">
+      <c r="A19" s="3">
         <v>18</v>
       </c>
-      <c r="B19" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C19" s="3" t="s">
+      <c r="B19" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C19" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="D19" s="3" t="s">
+      <c r="D19" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="E19" s="6" t="s">
+      <c r="E19" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="F19" s="3" t="s">
+      <c r="F19" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="G19" s="11">
+      <c r="G19" s="3">
         <v>2</v>
       </c>
     </row>
-    <row r="20" spans="1:7" ht="19.8" x14ac:dyDescent="0.45">
-      <c r="A20" s="11">
+    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="17.25">
+      <c r="A20" s="3">
         <v>19</v>
       </c>
-      <c r="B20" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C20" s="3" t="s">
+      <c r="B20" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C20" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="D20" s="3" t="s">
+      <c r="D20" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="E20" s="6" t="s">
+      <c r="E20" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="F20" s="3" t="s">
+      <c r="F20" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="G20" s="11">
+      <c r="G20" s="3">
         <v>2</v>
       </c>
     </row>
-    <row r="21" spans="1:7" ht="19.8" x14ac:dyDescent="0.45">
-      <c r="A21" s="11">
+    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="17.25">
+      <c r="A21" s="3">
         <v>20</v>
       </c>
-      <c r="B21" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C21" s="3" t="s">
+      <c r="B21" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C21" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="D21" s="3" t="s">
+      <c r="D21" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="E21" s="6" t="s">
+      <c r="E21" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="F21" s="3"/>
-      <c r="G21" s="11"/>
-    </row>
-    <row r="22" spans="1:7" ht="19.8" x14ac:dyDescent="0.45">
-      <c r="A22" s="11">
+      <c r="F21" s="4"/>
+      <c r="G21" s="3"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="17.25">
+      <c r="A22" s="3">
         <v>21</v>
       </c>
-      <c r="B22" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C22" s="3" t="s">
+      <c r="B22" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C22" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="D22" s="3" t="s">
+      <c r="D22" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="E22" s="6" t="s">
+      <c r="E22" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="F22" s="3"/>
-      <c r="G22" s="11"/>
-    </row>
-    <row r="23" spans="1:7" ht="19.8" x14ac:dyDescent="0.45">
-      <c r="A23" s="11">
+      <c r="F22" s="4"/>
+      <c r="G22" s="3"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="17.25">
+      <c r="A23" s="3">
         <v>22</v>
       </c>
-      <c r="B23" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C23" s="3" t="s">
+      <c r="B23" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C23" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="D23" s="3" t="s">
+      <c r="D23" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="E23" s="6" t="s">
+      <c r="E23" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="F23" s="3"/>
-      <c r="G23" s="11"/>
-    </row>
-    <row r="24" spans="1:7" ht="19.8" x14ac:dyDescent="0.45">
-      <c r="A24" s="11">
+      <c r="F23" s="4"/>
+      <c r="G23" s="3"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="17.25">
+      <c r="A24" s="3">
         <v>23</v>
       </c>
-      <c r="B24" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C24" s="3" t="s">
+      <c r="B24" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C24" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="D24" s="3" t="s">
+      <c r="D24" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="E24" s="6" t="s">
+      <c r="E24" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="F24" s="3"/>
-      <c r="G24" s="11"/>
+      <c r="F24" s="4"/>
+      <c r="G24" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Start Sliding Window Pattern
</commit_message>
<xml_diff>
--- a/7.Patterns Practice.xlsx
+++ b/7.Patterns Practice.xlsx
@@ -1,27 +1,28 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\samyak\learning\java\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD5C4569-1290-4BE7-BE77-A6EDAE9FD304}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D0F61F3-EE2D-4B21-9D35-86BB92AC2444}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Two Pointers" sheetId="1" r:id="rId1"/>
     <sheet name="Fast and Slow Pointers" sheetId="2" r:id="rId2"/>
+    <sheet name="Sliding Window" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="279" uniqueCount="129">
   <si>
     <t>No.</t>
   </si>
@@ -275,13 +276,148 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/reverse-string-ii/</t>
+  </si>
+  <si>
+    <t>Sliding Window</t>
+  </si>
+  <si>
+    <t>187. Repeated DNA Sequences</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/repeated-dna-sequences/</t>
+  </si>
+  <si>
+    <t>239. Sliding Window Maximum</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/sliding-window-maximum/</t>
+  </si>
+  <si>
+    <t>Minimum Window Subsequence</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/minimum-window-subsequence/description/</t>
+  </si>
+  <si>
+    <t>424. Longest Repeating Character Replacement</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/longest-repeating-character-replacement/</t>
+  </si>
+  <si>
+    <t>76. Minimum Window Substring</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/minimum-window-substring/</t>
+  </si>
+  <si>
+    <t>3. Longest Substring Without Repeating Characters</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/longest-substring-without-repeating-characters/</t>
+  </si>
+  <si>
+    <t>209. Minimum Size Subarray Sum</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/minimum-size-subarray-sum/</t>
+  </si>
+  <si>
+    <t>643. Maximum Average Subarray I</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/maximum-average-subarray-i/</t>
+  </si>
+  <si>
+    <t>1343. Number of Sub-arrays of Size K and Average Greater than or Equal to Threshold</t>
+  </si>
+  <si>
+    <t>MEDIUM</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/number-of-sub-arrays-of-size-k-and-average-greater-than-or-equal-to-threshold/description/</t>
+  </si>
+  <si>
+    <t>904. Fruit Into Baskets</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/fruit-into-baskets/</t>
+  </si>
+  <si>
+    <t>219. Contains Duplicate II</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/contains-duplicate-ii/</t>
+  </si>
+  <si>
+    <t>1838. Frequency of the Most Frequent Element</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/frequency-of-the-most-frequent-element/</t>
+  </si>
+  <si>
+    <t>992. Subarrays with K Different Integers</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/subarrays-with-k-different-integers/</t>
+  </si>
+  <si>
+    <t>2302. Count Subarrays With Score Less Than K</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/count-subarrays-with-score-less-than-k/</t>
+  </si>
+  <si>
+    <t>Count Substrings With K-Frequency Characters II</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/count-substrings-with-k-frequency-characters-ii/description/</t>
+  </si>
+  <si>
+    <t>2461. Maximum Sum of Distinct Subarrays With Length K</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/maximum-sum-of-distinct-subarrays-with-length-k/description/</t>
+  </si>
+  <si>
+    <t>Max Sum Subarray of size K</t>
+  </si>
+  <si>
+    <t>https://www.geeksforgeeks.org/problems/max-sum-subarray-of-size-k5313/1</t>
+  </si>
+  <si>
+    <t>Rabin Karp Algorithm</t>
+  </si>
+  <si>
+    <t>3. Longest Substring Without Repeating Characters (Map Approach)</t>
+  </si>
+  <si>
+    <t>HARD</t>
+  </si>
+  <si>
+    <t>Split a Linked List into two halves</t>
+  </si>
+  <si>
+    <t>https://www.geeksforgeeks.org/problems/split-a-circular-linked-list-into-two-halves/1</t>
+  </si>
+  <si>
+    <t>Unlock</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/reverse-words-in-a-string-iii/</t>
+  </si>
+  <si>
+    <t>557.Reverse Words in a String III</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -330,8 +466,27 @@
       <name val="Comic Sans MS"/>
       <family val="4"/>
     </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color rgb="FF000000"/>
+      <name val="Comic Sans MS"/>
+      <family val="4"/>
+    </font>
+    <font>
+      <sz val="13"/>
+      <color rgb="FF000000"/>
+      <name val="Comic Sans MS"/>
+      <family val="4"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -368,6 +523,24 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF00FF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF6600"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -415,7 +588,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -469,20 +642,73 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="7" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="8" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="8" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -493,8 +719,8 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FFFF6600"/>
       <color rgb="FFFF0066"/>
-      <color rgb="FFFF6600"/>
     </mruColors>
   </colors>
   <extLst>
@@ -796,7 +1022,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:G26"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5.6640625" style="11" bestFit="1" customWidth="1"/>
@@ -808,7 +1034,7 @@
     <col min="7" max="7" width="9.6640625" style="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:7" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -831,7 +1057,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:7" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A2" s="3">
         <v>1</v>
       </c>
@@ -854,7 +1080,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:7" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A3" s="3">
         <v>2</v>
       </c>
@@ -877,7 +1103,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:7" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A4" s="3">
         <v>3</v>
       </c>
@@ -900,7 +1126,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:7" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A5" s="3">
         <v>4</v>
       </c>
@@ -923,7 +1149,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:7" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A6" s="3">
         <v>5</v>
       </c>
@@ -946,7 +1172,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:7" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A7" s="3">
         <v>6</v>
       </c>
@@ -969,7 +1195,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:7" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A8" s="3">
         <v>7</v>
       </c>
@@ -1065,22 +1291,26 @@
       <c r="A12" s="3">
         <v>11</v>
       </c>
-      <c r="B12" s="16" t="s">
-        <v>7</v>
-      </c>
-      <c r="C12" s="16" t="s">
-        <v>29</v>
-      </c>
-      <c r="D12" s="16" t="s">
-        <v>30</v>
-      </c>
-      <c r="E12" s="17" t="s">
-        <v>31</v>
-      </c>
-      <c r="F12" s="16"/>
-      <c r="G12" s="15"/>
-    </row>
-    <row r="13" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B12" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G12" s="3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A13" s="3">
         <v>12</v>
       </c>
@@ -1088,18 +1318,18 @@
         <v>7</v>
       </c>
       <c r="C13" s="16" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="D13" s="16" t="s">
         <v>30</v>
       </c>
       <c r="E13" s="17" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="F13" s="16"/>
       <c r="G13" s="15"/>
     </row>
-    <row r="14" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:7" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A14" s="3">
         <v>13</v>
       </c>
@@ -1107,18 +1337,18 @@
         <v>7</v>
       </c>
       <c r="C14" s="16" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="D14" s="16" t="s">
         <v>30</v>
       </c>
       <c r="E14" s="17" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F14" s="16"/>
       <c r="G14" s="15"/>
     </row>
-    <row r="15" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:7" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A15" s="3">
         <v>14</v>
       </c>
@@ -1126,156 +1356,152 @@
         <v>7</v>
       </c>
       <c r="C15" s="16" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D15" s="16" t="s">
         <v>30</v>
       </c>
       <c r="E15" s="17" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="F15" s="16"/>
       <c r="G15" s="15"/>
     </row>
-    <row r="16" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:7" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A16" s="3">
         <v>15</v>
       </c>
-      <c r="B16" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="C16" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="D16" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="E16" s="14" t="s">
-        <v>40</v>
-      </c>
-      <c r="F16" s="7" t="s">
-        <v>59</v>
-      </c>
-      <c r="G16" s="13">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B16" s="16" t="s">
+        <v>7</v>
+      </c>
+      <c r="C16" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="D16" s="16" t="s">
+        <v>30</v>
+      </c>
+      <c r="E16" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="F16" s="16"/>
+      <c r="G16" s="15"/>
+    </row>
+    <row r="17" spans="1:7" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A17" s="3">
         <v>16</v>
       </c>
-      <c r="B17" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="C17" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="D17" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="E17" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="F17" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="G17" s="3">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B17" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C17" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="D17" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="E17" s="14" t="s">
+        <v>40</v>
+      </c>
+      <c r="F17" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="G17" s="13">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A18" s="3">
         <v>17</v>
       </c>
-      <c r="B18" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="C18" s="8" t="s">
-        <v>43</v>
-      </c>
-      <c r="D18" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="E18" s="9" t="s">
-        <v>44</v>
-      </c>
-      <c r="F18" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="G18" s="10" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B18" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E18" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="F18" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G18" s="3">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A19" s="3">
         <v>18</v>
       </c>
-      <c r="B19" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="C19" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="D19" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E19" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="F19" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="G19" s="3">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B19" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C19" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="D19" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="E19" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="F19" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="G19" s="10" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A20" s="3">
         <v>19</v>
       </c>
-      <c r="B20" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="C20" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="D20" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="E20" s="9" t="s">
-        <v>48</v>
-      </c>
-      <c r="F20" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="G20" s="10" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B20" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="E20" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="F20" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G20" s="3">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A21" s="3">
         <v>20</v>
       </c>
-      <c r="B21" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="C21" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="D21" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E21" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="F21" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="G21" s="3">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B21" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C21" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="D21" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="E21" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="F21" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="G21" s="10" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A22" s="3">
         <v>21</v>
       </c>
@@ -1283,22 +1509,22 @@
         <v>7</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="F22" s="4" t="s">
         <v>11</v>
       </c>
       <c r="G22" s="3">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.45">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A23" s="3">
         <v>22</v>
       </c>
@@ -1306,13 +1532,13 @@
         <v>7</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D23" s="4" t="s">
         <v>9</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="F23" s="4" t="s">
         <v>11</v>
@@ -1329,13 +1555,13 @@
         <v>7</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="D24" s="4" t="s">
         <v>9</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="F24" s="4" t="s">
         <v>11</v>
@@ -1352,18 +1578,41 @@
         <v>7</v>
       </c>
       <c r="C25" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D25" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E25" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="F25" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G25" s="3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A26" s="3">
+        <v>25</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C26" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="D25" s="4" t="s">
+      <c r="D26" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E25" s="5" t="s">
+      <c r="E26" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="F25" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="G25" s="3">
+      <c r="F26" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G26" s="3">
         <v>4</v>
       </c>
     </row>
@@ -1374,39 +1623,43 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6CFACA4C-4E46-4F7E-8751-AA8B53927209}">
-  <dimension ref="A1:F11"/>
-  <sheetFormatPr defaultRowHeight="19.8" x14ac:dyDescent="0.45"/>
+  <dimension ref="A1:G25"/>
+  <sheetFormatPr defaultRowHeight="19.8" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="5.6640625" style="21" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="27.6640625" style="21" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="49.88671875" style="21" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.109375" style="21" customWidth="1"/>
-    <col min="5" max="5" width="85.21875" style="21" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.44140625" style="21" customWidth="1"/>
-    <col min="7" max="16384" width="8.88671875" style="21"/>
+    <col min="1" max="1" width="5.6640625" style="33" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27.6640625" style="33" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="49.88671875" style="33" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.109375" style="33" customWidth="1"/>
+    <col min="5" max="5" width="85.21875" style="33" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.44140625" style="33" customWidth="1"/>
+    <col min="7" max="7" width="9.6640625" style="39" bestFit="1" customWidth="1"/>
+    <col min="8" max="16384" width="8.88671875" style="33"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="21" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A1" s="20" t="s">
+    <row r="1" spans="1:7" ht="41.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="31" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="20" t="s">
+      <c r="B1" s="31" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="20" t="s">
+      <c r="C1" s="31" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="20" t="s">
+      <c r="D1" s="31" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="20" t="s">
+      <c r="E1" s="31" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="20" t="s">
+      <c r="F1" s="31" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" ht="21" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="G1" s="35" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="21" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="18">
         <v>1</v>
       </c>
@@ -1422,9 +1675,14 @@
       <c r="E2" s="22" t="s">
         <v>63</v>
       </c>
-      <c r="F2" s="23"/>
-    </row>
-    <row r="3" spans="1:6" ht="21" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="F2" s="19" t="s">
+        <v>11</v>
+      </c>
+      <c r="G2" s="36">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="21" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="18">
         <v>2</v>
       </c>
@@ -1440,9 +1698,14 @@
       <c r="E3" s="22" t="s">
         <v>65</v>
       </c>
-      <c r="F3" s="23"/>
-    </row>
-    <row r="4" spans="1:6" ht="21" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="F3" s="19" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3" s="36">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="21" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="18">
         <v>3</v>
       </c>
@@ -1458,27 +1721,37 @@
       <c r="E4" s="22" t="s">
         <v>67</v>
       </c>
-      <c r="F4" s="23"/>
-    </row>
-    <row r="5" spans="1:6" ht="21" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A5" s="18">
+      <c r="F4" s="19" t="s">
+        <v>11</v>
+      </c>
+      <c r="G4" s="36">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="21" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="26">
         <v>4</v>
       </c>
-      <c r="B5" s="19" t="s">
+      <c r="B5" s="27" t="s">
         <v>61</v>
       </c>
-      <c r="C5" s="19" t="s">
+      <c r="C5" s="27" t="s">
         <v>68</v>
       </c>
-      <c r="D5" s="19" t="s">
+      <c r="D5" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="E5" s="22" t="s">
+      <c r="E5" s="28" t="s">
         <v>69</v>
       </c>
-      <c r="F5" s="23"/>
-    </row>
-    <row r="6" spans="1:6" ht="21" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="F5" s="27" t="s">
+        <v>126</v>
+      </c>
+      <c r="G5" s="37">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="21" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="18">
         <v>5</v>
       </c>
@@ -1494,9 +1767,14 @@
       <c r="E6" s="22" t="s">
         <v>71</v>
       </c>
-      <c r="F6" s="23"/>
-    </row>
-    <row r="7" spans="1:6" ht="21" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="F6" s="19" t="s">
+        <v>11</v>
+      </c>
+      <c r="G6" s="36">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="21" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="18">
         <v>6</v>
       </c>
@@ -1512,9 +1790,14 @@
       <c r="E7" s="22" t="s">
         <v>73</v>
       </c>
-      <c r="F7" s="23"/>
-    </row>
-    <row r="8" spans="1:6" ht="21" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="F7" s="19" t="s">
+        <v>11</v>
+      </c>
+      <c r="G7" s="36">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="21" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="18">
         <v>7</v>
       </c>
@@ -1530,27 +1813,37 @@
       <c r="E8" s="22" t="s">
         <v>75</v>
       </c>
-      <c r="F8" s="23"/>
-    </row>
-    <row r="9" spans="1:6" ht="21" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A9" s="18">
+      <c r="F8" s="19" t="s">
+        <v>11</v>
+      </c>
+      <c r="G8" s="36">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="21" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="29">
         <v>8</v>
       </c>
-      <c r="B9" s="19" t="s">
+      <c r="B9" s="30" t="s">
         <v>61</v>
       </c>
-      <c r="C9" s="19" t="s">
+      <c r="C9" s="30" t="s">
         <v>76</v>
       </c>
-      <c r="D9" s="18" t="s">
+      <c r="D9" s="29" t="s">
         <v>39</v>
       </c>
-      <c r="E9" s="22" t="s">
+      <c r="E9" s="34" t="s">
         <v>77</v>
       </c>
-      <c r="F9" s="23"/>
-    </row>
-    <row r="10" spans="1:6" ht="21" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="F9" s="30" t="s">
+        <v>125</v>
+      </c>
+      <c r="G9" s="38" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="21" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="18">
         <v>9</v>
       </c>
@@ -1566,9 +1859,14 @@
       <c r="E10" s="22" t="s">
         <v>79</v>
       </c>
-      <c r="F10" s="23"/>
-    </row>
-    <row r="11" spans="1:6" ht="21" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="F10" s="19" t="s">
+        <v>11</v>
+      </c>
+      <c r="G10" s="36">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="21" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="18">
         <v>10</v>
       </c>
@@ -1584,9 +1882,59 @@
       <c r="E11" s="22" t="s">
         <v>81</v>
       </c>
-      <c r="F11" s="23"/>
-    </row>
+      <c r="F11" s="19" t="s">
+        <v>11</v>
+      </c>
+      <c r="G11" s="36">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="40.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="18">
+        <v>11</v>
+      </c>
+      <c r="B12" s="19" t="s">
+        <v>61</v>
+      </c>
+      <c r="C12" s="19" t="s">
+        <v>123</v>
+      </c>
+      <c r="D12" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="E12" s="22" t="s">
+        <v>124</v>
+      </c>
+      <c r="F12" s="19" t="s">
+        <v>11</v>
+      </c>
+      <c r="G12" s="36">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="G13" s="33"/>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="G14" s="33"/>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="G15" s="33"/>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="G16" s="33"/>
+    </row>
+    <row r="17" s="33" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="18" s="33" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="19" s="33" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="20" s="33" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="21" s="33" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="22" s="33" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="23" s="33" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="24" s="33" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="25" s="33" customFormat="1" x14ac:dyDescent="0.3"/>
   </sheetData>
+  <phoneticPr fontId="9" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="E2" r:id="rId1" xr:uid="{4E66C6E8-32CD-4460-BFF3-BD29EA0C5AFF}"/>
     <hyperlink ref="E3" r:id="rId2" xr:uid="{133791DF-AAD5-42EB-9410-96B0FAA8FB85}"/>
@@ -1598,6 +1946,459 @@
     <hyperlink ref="E9" r:id="rId8" xr:uid="{92E14B6B-C171-499C-AA12-4DE7BCC227DD}"/>
     <hyperlink ref="E10" r:id="rId9" xr:uid="{293BD634-5303-4800-BFAF-6FF9F43F60A6}"/>
     <hyperlink ref="E11" r:id="rId10" xr:uid="{CD16331C-7203-4637-8A8B-42BB612AE110}"/>
+    <hyperlink ref="E12" r:id="rId11" xr:uid="{26BBD6BD-A369-4011-BD53-A0D7F84193D6}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D2AB2C82-5D2F-4E18-ADA4-8FB538DDE1AD}">
+  <dimension ref="A1:G25"/>
+  <sheetFormatPr defaultRowHeight="19.8" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="5.6640625" style="33" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.88671875" style="33" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="65.44140625" style="33" customWidth="1"/>
+    <col min="4" max="4" width="11.88671875" style="33" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="84.77734375" style="33" customWidth="1"/>
+    <col min="6" max="6" width="7" style="33" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.77734375" style="39" bestFit="1" customWidth="1"/>
+    <col min="8" max="16384" width="8.88671875" style="33"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" s="40" customFormat="1" ht="21" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="31" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="31" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="31" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="31" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="31" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="31" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="35" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="20.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="19">
+        <v>1</v>
+      </c>
+      <c r="B2" s="19" t="s">
+        <v>84</v>
+      </c>
+      <c r="C2" s="19" t="s">
+        <v>85</v>
+      </c>
+      <c r="D2" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="E2" s="22" t="s">
+        <v>86</v>
+      </c>
+      <c r="F2" s="19"/>
+      <c r="G2" s="36"/>
+    </row>
+    <row r="3" spans="1:7" ht="20.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="20">
+        <v>2</v>
+      </c>
+      <c r="B3" s="20" t="s">
+        <v>84</v>
+      </c>
+      <c r="C3" s="20" t="s">
+        <v>87</v>
+      </c>
+      <c r="D3" s="20" t="s">
+        <v>30</v>
+      </c>
+      <c r="E3" s="23" t="s">
+        <v>88</v>
+      </c>
+      <c r="F3" s="20"/>
+      <c r="G3" s="20"/>
+    </row>
+    <row r="4" spans="1:7" ht="40.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="21">
+        <v>3</v>
+      </c>
+      <c r="B4" s="21" t="s">
+        <v>84</v>
+      </c>
+      <c r="C4" s="21" t="s">
+        <v>89</v>
+      </c>
+      <c r="D4" s="21" t="s">
+        <v>39</v>
+      </c>
+      <c r="E4" s="24" t="s">
+        <v>90</v>
+      </c>
+      <c r="F4" s="21"/>
+      <c r="G4" s="21"/>
+    </row>
+    <row r="5" spans="1:7" ht="40.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="19">
+        <v>4</v>
+      </c>
+      <c r="B5" s="19" t="s">
+        <v>84</v>
+      </c>
+      <c r="C5" s="19" t="s">
+        <v>91</v>
+      </c>
+      <c r="D5" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="E5" s="22" t="s">
+        <v>92</v>
+      </c>
+      <c r="F5" s="19"/>
+      <c r="G5" s="36"/>
+    </row>
+    <row r="6" spans="1:7" ht="20.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="32">
+        <v>5</v>
+      </c>
+      <c r="B6" s="32" t="s">
+        <v>84</v>
+      </c>
+      <c r="C6" s="32" t="s">
+        <v>93</v>
+      </c>
+      <c r="D6" s="32" t="s">
+        <v>30</v>
+      </c>
+      <c r="E6" s="25" t="s">
+        <v>94</v>
+      </c>
+      <c r="F6" s="32"/>
+      <c r="G6" s="32"/>
+    </row>
+    <row r="7" spans="1:7" ht="40.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="19">
+        <v>6</v>
+      </c>
+      <c r="B7" s="19" t="s">
+        <v>84</v>
+      </c>
+      <c r="C7" s="19" t="s">
+        <v>95</v>
+      </c>
+      <c r="D7" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="E7" s="22" t="s">
+        <v>96</v>
+      </c>
+      <c r="F7" s="19"/>
+      <c r="G7" s="36"/>
+    </row>
+    <row r="8" spans="1:7" ht="20.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="19">
+        <v>7</v>
+      </c>
+      <c r="B8" s="19" t="s">
+        <v>84</v>
+      </c>
+      <c r="C8" s="19" t="s">
+        <v>97</v>
+      </c>
+      <c r="D8" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="E8" s="22" t="s">
+        <v>98</v>
+      </c>
+      <c r="F8" s="19" t="s">
+        <v>11</v>
+      </c>
+      <c r="G8" s="36">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="20.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="19">
+        <v>8</v>
+      </c>
+      <c r="B9" s="19" t="s">
+        <v>84</v>
+      </c>
+      <c r="C9" s="19" t="s">
+        <v>99</v>
+      </c>
+      <c r="D9" s="19" t="s">
+        <v>9</v>
+      </c>
+      <c r="E9" s="22" t="s">
+        <v>100</v>
+      </c>
+      <c r="F9" s="19"/>
+      <c r="G9" s="36"/>
+    </row>
+    <row r="10" spans="1:7" ht="40.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="19">
+        <v>9</v>
+      </c>
+      <c r="B10" s="19" t="s">
+        <v>84</v>
+      </c>
+      <c r="C10" s="19" t="s">
+        <v>101</v>
+      </c>
+      <c r="D10" s="19" t="s">
+        <v>102</v>
+      </c>
+      <c r="E10" s="22" t="s">
+        <v>103</v>
+      </c>
+      <c r="F10" s="19"/>
+      <c r="G10" s="36"/>
+    </row>
+    <row r="11" spans="1:7" ht="20.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="19">
+        <v>10</v>
+      </c>
+      <c r="B11" s="19" t="s">
+        <v>84</v>
+      </c>
+      <c r="C11" s="19" t="s">
+        <v>104</v>
+      </c>
+      <c r="D11" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="E11" s="22" t="s">
+        <v>105</v>
+      </c>
+      <c r="F11" s="19"/>
+      <c r="G11" s="36"/>
+    </row>
+    <row r="12" spans="1:7" ht="20.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="19">
+        <v>11</v>
+      </c>
+      <c r="B12" s="19" t="s">
+        <v>84</v>
+      </c>
+      <c r="C12" s="19" t="s">
+        <v>106</v>
+      </c>
+      <c r="D12" s="19" t="s">
+        <v>9</v>
+      </c>
+      <c r="E12" s="22" t="s">
+        <v>107</v>
+      </c>
+      <c r="F12" s="19"/>
+      <c r="G12" s="36"/>
+    </row>
+    <row r="13" spans="1:7" ht="40.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="19">
+        <v>12</v>
+      </c>
+      <c r="B13" s="19" t="s">
+        <v>84</v>
+      </c>
+      <c r="C13" s="19" t="s">
+        <v>108</v>
+      </c>
+      <c r="D13" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="E13" s="22" t="s">
+        <v>109</v>
+      </c>
+      <c r="F13" s="19"/>
+      <c r="G13" s="36"/>
+    </row>
+    <row r="14" spans="1:7" ht="20.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="32">
+        <v>13</v>
+      </c>
+      <c r="B14" s="32" t="s">
+        <v>84</v>
+      </c>
+      <c r="C14" s="32" t="s">
+        <v>110</v>
+      </c>
+      <c r="D14" s="32" t="s">
+        <v>30</v>
+      </c>
+      <c r="E14" s="25" t="s">
+        <v>111</v>
+      </c>
+      <c r="F14" s="32"/>
+      <c r="G14" s="32"/>
+    </row>
+    <row r="15" spans="1:7" ht="40.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="32">
+        <v>14</v>
+      </c>
+      <c r="B15" s="32" t="s">
+        <v>84</v>
+      </c>
+      <c r="C15" s="32" t="s">
+        <v>112</v>
+      </c>
+      <c r="D15" s="32" t="s">
+        <v>30</v>
+      </c>
+      <c r="E15" s="25" t="s">
+        <v>113</v>
+      </c>
+      <c r="F15" s="32"/>
+      <c r="G15" s="32"/>
+    </row>
+    <row r="16" spans="1:7" ht="40.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="32">
+        <v>15</v>
+      </c>
+      <c r="B16" s="20" t="s">
+        <v>84</v>
+      </c>
+      <c r="C16" s="20" t="s">
+        <v>114</v>
+      </c>
+      <c r="D16" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="E16" s="23" t="s">
+        <v>115</v>
+      </c>
+      <c r="F16" s="20"/>
+      <c r="G16" s="32"/>
+    </row>
+    <row r="17" spans="1:7" ht="40.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="19">
+        <v>16</v>
+      </c>
+      <c r="B17" s="19" t="s">
+        <v>84</v>
+      </c>
+      <c r="C17" s="19" t="s">
+        <v>116</v>
+      </c>
+      <c r="D17" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="E17" s="22" t="s">
+        <v>117</v>
+      </c>
+      <c r="F17" s="19" t="s">
+        <v>11</v>
+      </c>
+      <c r="G17" s="36">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="40.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="19">
+        <v>17</v>
+      </c>
+      <c r="B18" s="19" t="s">
+        <v>84</v>
+      </c>
+      <c r="C18" s="19" t="s">
+        <v>118</v>
+      </c>
+      <c r="D18" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="E18" s="22" t="s">
+        <v>119</v>
+      </c>
+      <c r="F18" s="19" t="s">
+        <v>11</v>
+      </c>
+      <c r="G18" s="36">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="20.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="19">
+        <v>18</v>
+      </c>
+      <c r="B19" s="19" t="s">
+        <v>84</v>
+      </c>
+      <c r="C19" s="19" t="s">
+        <v>120</v>
+      </c>
+      <c r="D19" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="E19" s="22" t="s">
+        <v>86</v>
+      </c>
+      <c r="F19" s="19"/>
+      <c r="G19" s="36"/>
+    </row>
+    <row r="20" spans="1:7" ht="40.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="19">
+        <v>19</v>
+      </c>
+      <c r="B20" s="19" t="s">
+        <v>84</v>
+      </c>
+      <c r="C20" s="19" t="s">
+        <v>121</v>
+      </c>
+      <c r="D20" s="19" t="s">
+        <v>122</v>
+      </c>
+      <c r="E20" s="22" t="s">
+        <v>96</v>
+      </c>
+      <c r="F20" s="19"/>
+      <c r="G20" s="36"/>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="G21" s="33"/>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="G22" s="33"/>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="G23" s="33"/>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="G24" s="33"/>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="G25" s="33"/>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="E2" r:id="rId1" xr:uid="{6EC5FB5A-5B4A-4E53-9032-DF651B49380F}"/>
+    <hyperlink ref="E3" r:id="rId2" xr:uid="{AE51BFE8-DE9F-404A-8B28-0A37CB7C5249}"/>
+    <hyperlink ref="E4" r:id="rId3" xr:uid="{AE3E90E6-A32D-4E19-99D2-F382983DE985}"/>
+    <hyperlink ref="E5" r:id="rId4" xr:uid="{7292E66B-1BD7-48CC-9099-9EBCB5716E0F}"/>
+    <hyperlink ref="E6" r:id="rId5" xr:uid="{9B1A21F1-E3A3-4914-B5C7-A89181BB976F}"/>
+    <hyperlink ref="E7" r:id="rId6" xr:uid="{E5FF4577-5164-4B07-B55E-FC83FF5FC660}"/>
+    <hyperlink ref="E8" r:id="rId7" xr:uid="{948A650F-1BC2-4E5B-ADA3-BB4055DD088D}"/>
+    <hyperlink ref="E9" r:id="rId8" xr:uid="{A9C23591-B4C7-402A-88C6-9301464C0E24}"/>
+    <hyperlink ref="E10" r:id="rId9" xr:uid="{B6B64FC8-69C9-4874-8D7D-C634ABFF6758}"/>
+    <hyperlink ref="E11" r:id="rId10" xr:uid="{B0B29EFD-9999-4413-AA64-FC8BB822D05C}"/>
+    <hyperlink ref="E12" r:id="rId11" xr:uid="{7BB83799-3EF8-4081-83DB-70ED31977076}"/>
+    <hyperlink ref="E13" r:id="rId12" xr:uid="{F26FE565-EC47-47BE-B575-19D9F9AB3C87}"/>
+    <hyperlink ref="E14" r:id="rId13" xr:uid="{C2E57023-CDF4-4F60-91A0-CC84749B30AC}"/>
+    <hyperlink ref="E15" r:id="rId14" xr:uid="{1A69F66B-1300-4D51-B35E-F0FCA666C3EC}"/>
+    <hyperlink ref="E16" r:id="rId15" xr:uid="{426743A7-B655-4339-BFD0-2869570BBC4A}"/>
+    <hyperlink ref="E17" r:id="rId16" xr:uid="{CB41EABC-5D79-417B-AFAA-C217764882F8}"/>
+    <hyperlink ref="E18" r:id="rId17" xr:uid="{7B1E49EA-CB7C-4FDE-9F19-1DBA346C2394}"/>
+    <hyperlink ref="E19" r:id="rId18" xr:uid="{471D3E92-6E98-4C2A-85C6-97D099BD326C}"/>
+    <hyperlink ref="E20" r:id="rId19" xr:uid="{607D06C9-E5D5-4E55-BAED-12A1F5471C15}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>